<commit_message>
fix: fixed blockages in export sheet
</commit_message>
<xml_diff>
--- a/Database_to_Dashboard_Mapping.xlsx
+++ b/Database_to_Dashboard_Mapping.xlsx
@@ -4031,12 +4031,12 @@
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>coronary_angiogram_done, single_vessel_disease, double_vessel_disease, triple_vessel_disease, left_main_disease</t>
+          <t>ecg_lbbb, ecg_rbbb, ecg_block_other, ecg_block_other_details</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t>VARCHAR(20)</t>
+          <t>VARCHAR(50)</t>
         </is>
       </c>
       <c r="G59" s="10" t="inlineStr">
@@ -4046,7 +4046,7 @@
       </c>
       <c r="H59" s="9" t="inlineStr">
         <is>
-          <t>CASE WHEN 'Yes' IN (single_vessel_disease, double_vessel_disease, triple_vessel_disease, left_main_disease) THEN 'Yes' ELSE 'No' END</t>
+          <t>CASE WHEN ecg_lbbb = 'Yes' THEN 'lbbb' WHEN ecg_rbbb = 'Yes' THEN 'rbbb' WHEN ecg_block_other = 'Yes' THEN COALESCE(ecg_block_other_details, 'Other') ELSE 'No' END</t>
         </is>
       </c>
       <c r="I59" s="9" t="inlineStr">
@@ -4056,7 +4056,7 @@
       </c>
       <c r="J59" s="8" t="inlineStr">
         <is>
-          <t>Coronary angiographic documentation of epicardial stenosis</t>
+          <t>Presence of ECG conduction blockages (lbbb, rbbb, or ecg_block_other_details)</t>
         </is>
       </c>
     </row>

</xml_diff>